<commit_message>
add lignes in excel BDD
</commit_message>
<xml_diff>
--- a/backend/processing/fixtures/processing_templates.xlsx
+++ b/backend/processing/fixtures/processing_templates.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:H243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7134,7 +7134,7 @@
         </is>
       </c>
     </row>
-    <row r="166">
+    <row r="166" ht="99" customHeight="1">
       <c r="A166" s="4" t="n">
         <v>165</v>
       </c>
@@ -7174,7 +7174,7 @@
         </is>
       </c>
     </row>
-    <row r="167">
+    <row r="167" ht="73" customHeight="1">
       <c r="A167" s="4" t="n">
         <v>166</v>
       </c>
@@ -7214,7 +7214,7 @@
         </is>
       </c>
     </row>
-    <row r="168">
+    <row r="168" ht="73" customHeight="1">
       <c r="A168" s="4" t="n">
         <v>167</v>
       </c>
@@ -7254,7 +7254,7 @@
         </is>
       </c>
     </row>
-    <row r="169">
+    <row r="169" ht="60" customHeight="1">
       <c r="A169" s="4" t="n">
         <v>168</v>
       </c>
@@ -7294,7 +7294,7 @@
         </is>
       </c>
     </row>
-    <row r="170">
+    <row r="170" ht="73" customHeight="1">
       <c r="A170" s="4" t="n">
         <v>169</v>
       </c>
@@ -7334,7 +7334,7 @@
         </is>
       </c>
     </row>
-    <row r="171">
+    <row r="171" ht="73" customHeight="1">
       <c r="A171" s="4" t="n">
         <v>170</v>
       </c>
@@ -7374,7 +7374,7 @@
         </is>
       </c>
     </row>
-    <row r="172">
+    <row r="172" ht="86" customHeight="1">
       <c r="A172" s="4" t="n">
         <v>171</v>
       </c>
@@ -7414,7 +7414,7 @@
         </is>
       </c>
     </row>
-    <row r="173">
+    <row r="173" ht="99" customHeight="1">
       <c r="A173" s="4" t="n">
         <v>172</v>
       </c>
@@ -7454,7 +7454,7 @@
         </is>
       </c>
     </row>
-    <row r="174">
+    <row r="174" ht="45" customHeight="1">
       <c r="A174" s="4" t="n">
         <v>173</v>
       </c>
@@ -7494,7 +7494,7 @@
         </is>
       </c>
     </row>
-    <row r="175">
+    <row r="175" ht="112" customHeight="1">
       <c r="A175" s="4" t="n">
         <v>174</v>
       </c>
@@ -7534,7 +7534,7 @@
         </is>
       </c>
     </row>
-    <row r="176">
+    <row r="176" ht="47" customHeight="1">
       <c r="A176" s="4" t="n">
         <v>175</v>
       </c>
@@ -7574,7 +7574,7 @@
         </is>
       </c>
     </row>
-    <row r="177">
+    <row r="177" ht="112" customHeight="1">
       <c r="A177" s="4" t="n">
         <v>176</v>
       </c>
@@ -7614,7 +7614,7 @@
         </is>
       </c>
     </row>
-    <row r="178">
+    <row r="178" ht="151" customHeight="1">
       <c r="A178" s="4" t="n">
         <v>177</v>
       </c>
@@ -7654,7 +7654,7 @@
         </is>
       </c>
     </row>
-    <row r="179">
+    <row r="179" ht="216" customHeight="1">
       <c r="A179" s="4" t="n">
         <v>178</v>
       </c>
@@ -7694,7 +7694,7 @@
         </is>
       </c>
     </row>
-    <row r="180">
+    <row r="180" ht="151" customHeight="1">
       <c r="A180" s="4" t="n">
         <v>179</v>
       </c>
@@ -7734,7 +7734,7 @@
         </is>
       </c>
     </row>
-    <row r="181">
+    <row r="181" ht="164" customHeight="1">
       <c r="A181" s="4" t="n">
         <v>180</v>
       </c>
@@ -7774,7 +7774,7 @@
         </is>
       </c>
     </row>
-    <row r="182">
+    <row r="182" ht="138" customHeight="1">
       <c r="A182" s="4" t="n">
         <v>181</v>
       </c>
@@ -7814,7 +7814,7 @@
         </is>
       </c>
     </row>
-    <row r="183">
+    <row r="183" ht="112" customHeight="1">
       <c r="A183" s="4" t="n">
         <v>182</v>
       </c>
@@ -7854,7 +7854,7 @@
         </is>
       </c>
     </row>
-    <row r="184">
+    <row r="184" ht="99" customHeight="1">
       <c r="A184" s="4" t="n">
         <v>183</v>
       </c>
@@ -7894,7 +7894,7 @@
         </is>
       </c>
     </row>
-    <row r="185">
+    <row r="185" ht="138" customHeight="1">
       <c r="A185" s="4" t="n">
         <v>184</v>
       </c>
@@ -7934,7 +7934,7 @@
         </is>
       </c>
     </row>
-    <row r="186">
+    <row r="186" ht="47" customHeight="1">
       <c r="A186" s="4" t="n">
         <v>185</v>
       </c>
@@ -7974,7 +7974,7 @@
         </is>
       </c>
     </row>
-    <row r="187">
+    <row r="187" ht="86" customHeight="1">
       <c r="A187" s="4" t="n">
         <v>186</v>
       </c>
@@ -8009,6 +8009,2246 @@
         </is>
       </c>
       <c r="H187" s="5" t="inlineStr">
+        <is>
+          <t>120 شهر (10 سنوات) / 120 mois (10 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="47" customHeight="1">
+      <c r="A188" s="4" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" s="5" t="inlineStr">
+        <is>
+          <t>أشغال عمومية / Travaux publics</t>
+        </is>
+      </c>
+      <c r="C188" s="5" t="inlineStr">
+        <is>
+          <t>إدارة حضور العمال / Gestion de la présence des travailleurs</t>
+        </is>
+      </c>
+      <c r="D188" s="5" t="inlineStr">
+        <is>
+          <t>متابعة ومراقبة حضور العمال / Suivi et contrôle de la présence des travailleurs</t>
+        </is>
+      </c>
+      <c r="E188" s="5" t="inlineStr">
+        <is>
+          <t>تسيير حضور الموظفين / Gestion de la présence des employés</t>
+        </is>
+      </c>
+      <c r="F188" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء، المتمهنون / Salariés, apprentis</t>
+        </is>
+      </c>
+      <c r="G188" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، الوظيفة، رقم التسجيل / Nom et prénom, fonction, matricule</t>
+        </is>
+      </c>
+      <c r="H188" s="5" t="inlineStr">
+        <is>
+          <t>36 شهر (03 سنوات) / 36 mois (3 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="99" customHeight="1">
+      <c r="A189" s="4" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" s="5" t="inlineStr">
+        <is>
+          <t>أشغال عمومية / Travaux publics</t>
+        </is>
+      </c>
+      <c r="C189" s="5" t="inlineStr">
+        <is>
+          <t>طب العمل / Médecine du travail</t>
+        </is>
+      </c>
+      <c r="D189" s="5" t="inlineStr">
+        <is>
+          <t>مراقبة الحالة الصحية للعمال والمتمهنين عن طريق إجراء فحوص طبية دورية وإجراء تقييم الكفاءة في العمل / Surveillance de l'état de santé des travailleurs et des apprentis par des examens médicaux périodiques et l'évaluation de l'aptitude au travail</t>
+        </is>
+      </c>
+      <c r="E189" s="5" t="inlineStr">
+        <is>
+          <t>طب العمل / Médecine du travail</t>
+        </is>
+      </c>
+      <c r="F189" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء، المتمهنون / Salariés, apprentis</t>
+        </is>
+      </c>
+      <c r="G189" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، تاريخ ومكان الازدياد، الحالة العائلية، عنوان السكن، عنوان البريد الإلكتروني، رقم الهاتف، الوظيفة، تقرير الصحة المهنية / Nom et prénom, date et lieu de naissance, situation familiale, adresse, e-mail, téléphone, fonction, rapport de santé au travail</t>
+        </is>
+      </c>
+      <c r="H189" s="5" t="inlineStr">
+        <is>
+          <t>36 شهر (03 سنوات) / 36 mois (3 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="60" customHeight="1">
+      <c r="A190" s="4" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" s="5" t="inlineStr">
+        <is>
+          <t>أشغال عمومية / Travaux publics</t>
+        </is>
+      </c>
+      <c r="C190" s="5" t="inlineStr">
+        <is>
+          <t>تسيير كاميرات المراقبة / Gestion des caméras de surveillance</t>
+        </is>
+      </c>
+      <c r="D190" s="5" t="inlineStr">
+        <is>
+          <t>مراقبة أماكن العمل / Surveillance des lieux de travail</t>
+        </is>
+      </c>
+      <c r="E190" s="5" t="inlineStr">
+        <is>
+          <t>تسيير تواجد الكاميرات / Gestion de la présence des caméras</t>
+        </is>
+      </c>
+      <c r="F190" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء، الموردون، الزبائن الحاليون أو المحتملون، الزوار / Salariés, fournisseurs, clients actuels ou potentiels, visiteurs</t>
+        </is>
+      </c>
+      <c r="G190" s="5" t="inlineStr">
+        <is>
+          <t>صورة في الفيديو / Image vidéo</t>
+        </is>
+      </c>
+      <c r="H190" s="5" t="inlineStr">
+        <is>
+          <t>شهر واحد / 1 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="86" customHeight="1">
+      <c r="A191" s="4" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>الاتصالات والمواصلات عبر الأقمار الصناعية / Télécommunications et communications par satellite</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>مراقبة الدخول / Contrôle des accès</t>
+        </is>
+      </c>
+      <c r="D191" s="5" t="inlineStr">
+        <is>
+          <t>مراقبة الدخول لضمان سلامة الممتلكات والأشخاص / Contrôle des accès pour assurer la sécurité des biens et des personnes</t>
+        </is>
+      </c>
+      <c r="E191" s="5" t="inlineStr">
+        <is>
+          <t>الأمن ومراقبة الدخول / Sécurité et contrôle des accès</t>
+        </is>
+      </c>
+      <c r="F191" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء، الموردون، الزبائن الحاليون أو المحتملون، المترشحون، المتمهنون، المتربصون وزوار آخرون / Salariés, fournisseurs, clients actuels ou potentiels, candidats, apprentis, stagiaires et autres visiteurs</t>
+        </is>
+      </c>
+      <c r="G191" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، رقم وثيقة الهوية/رخصة السياقة/جواز السفر، ترقيم السيارة، نسخة من جواز سفر أجنبي / Nom et prénom, n° CNI/permis de conduire/passeport, immatriculation du véhicule, copie de passeport étranger</t>
+        </is>
+      </c>
+      <c r="H191" s="5" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="112" customHeight="1">
+      <c r="A192" s="4" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" s="5" t="inlineStr">
+        <is>
+          <t>أشغال الطرق / Travaux routiers</t>
+        </is>
+      </c>
+      <c r="C192" s="5" t="inlineStr">
+        <is>
+          <t>السجلات القانونية / Registres légaux</t>
+        </is>
+      </c>
+      <c r="D192" s="5" t="inlineStr">
+        <is>
+          <t>تحديث بيانات العمال في السجلات القانونية للمؤسسة / Mise à jour des données des travailleurs dans les registres légaux de l'entreprise</t>
+        </is>
+      </c>
+      <c r="E192" s="5" t="inlineStr">
+        <is>
+          <t>تسيير السجلات القانونية / Gestion des registres légaux</t>
+        </is>
+      </c>
+      <c r="F192" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G192" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، تاريخ ومكان الازدياد، عنوان السكن، رقم الضمان الاجتماعي، الوظيفة، الجنس، طبيعة علاقة العمل، مدة العطلة، تاريخ التوظيف، تاريخ انتهاء علاقة العمل، الدخل / Nom et prénom, date et lieu de naissance, adresse, n° sécurité sociale, fonction, sexe, nature de la relation de travail, durée de congé, date de recrutement, date de fin de la relation de travail, revenu</t>
+        </is>
+      </c>
+      <c r="H192" s="5" t="inlineStr">
+        <is>
+          <t>384 شهر (32 سنة) / 384 mois (32 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="60" customHeight="1">
+      <c r="A193" s="4" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>أشغال الطرق / Travaux routiers</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>تسيير الزبائن / Gestion des clients</t>
+        </is>
+      </c>
+      <c r="D193" s="5" t="inlineStr">
+        <is>
+          <t>المتابعة التجارية لملفات الزبائن / Suivi commercial des dossiers clients</t>
+        </is>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>تسيير الزبائن / Gestion des clients</t>
+        </is>
+      </c>
+      <c r="F193" s="5" t="inlineStr">
+        <is>
+          <t>الزبائن الحاليون أو المحتملون / Clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G193" s="5" t="inlineStr">
+        <is>
+          <t>رقم التعريف الوطني، الاسم واللقب، عنوان البريد الإلكتروني، رقم الهاتف، التسمية الاجتماعية، البنك، رقم الحساب البنكي / NIN, nom et prénom, e-mail, téléphone, dénomination sociale, banque, n° compte bancaire</t>
+        </is>
+      </c>
+      <c r="H193" s="5" t="inlineStr">
+        <is>
+          <t>120 شهر (10 سنوات) / 120 mois (10 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="47" customHeight="1">
+      <c r="A194" s="4" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" s="5" t="inlineStr">
+        <is>
+          <t>أشغال الطرق / Travaux routiers</t>
+        </is>
+      </c>
+      <c r="C194" s="5" t="inlineStr">
+        <is>
+          <t>إدارة الحضور / Gestion de la présence</t>
+        </is>
+      </c>
+      <c r="D194" s="5" t="inlineStr">
+        <is>
+          <t>مراقبة ومتابعة الحضور / Contrôle et suivi de la présence</t>
+        </is>
+      </c>
+      <c r="E194" s="5" t="inlineStr">
+        <is>
+          <t>تسيير حضور الموظفين / Gestion de la présence des employés</t>
+        </is>
+      </c>
+      <c r="F194" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء، المتمهنون/المتربصون / Salariés, apprentis/stagiaires</t>
+        </is>
+      </c>
+      <c r="G194" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، صورة، معطيات بيومترية (الأصبع والوجه)، رقم التسجيل / Nom et prénom, photo, données biométriques (empreinte digitale et visage), matricule</t>
+        </is>
+      </c>
+      <c r="H194" s="5" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="73" customHeight="1">
+      <c r="A195" s="4" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" s="5" t="inlineStr">
+        <is>
+          <t>أشغال الطرق / Travaux routiers</t>
+        </is>
+      </c>
+      <c r="C195" s="5" t="inlineStr">
+        <is>
+          <t>معالجة النزاعات والاستشارات القانونية / Traitement des litiges et consultations juridiques</t>
+        </is>
+      </c>
+      <c r="D195" s="5" t="inlineStr">
+        <is>
+          <t>تسيير قضايا المنازعات والاستشارات القانونية / Gestion des affaires contentieuses et des consultations juridiques</t>
+        </is>
+      </c>
+      <c r="E195" s="5" t="inlineStr">
+        <is>
+          <t>تسيير النزاعات والاستشارات القانونية / Gestion des litiges et consultations juridiques</t>
+        </is>
+      </c>
+      <c r="F195" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء، ممثلو الشركات المتعاقدة مع المؤسسة / Salariés, représentants des sociétés contractantes avec l'entreprise</t>
+        </is>
+      </c>
+      <c r="G195" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، تاريخ ومكان الازدياد، الحالة العائلية، عنوان السكن، الجنس، عقد العمل، رقم الحساب البنكي/البريدي / Nom et prénom, date et lieu de naissance, situation familiale, adresse, sexe, contrat de travail, n° compte bancaire/postal</t>
+        </is>
+      </c>
+      <c r="H195" s="5" t="inlineStr">
+        <is>
+          <t>120 شهر (10 سنوات) / 120 mois (10 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="86" customHeight="1">
+      <c r="A196" s="4" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" s="5" t="inlineStr">
+        <is>
+          <t>أشغال الطرق / Travaux routiers</t>
+        </is>
+      </c>
+      <c r="C196" s="5" t="inlineStr">
+        <is>
+          <t>إدارة الموردين ومقدمي الخدمات / Gestion des fournisseurs et prestataires de services</t>
+        </is>
+      </c>
+      <c r="D196" s="5" t="inlineStr">
+        <is>
+          <t>إدارة العلاقات مع الموردين ومقدمي الخدمات - الإدارة التجارية وإعداد الفواتير / Gestion des relations avec les fournisseurs et prestataires de services - administration commerciale et facturation</t>
+        </is>
+      </c>
+      <c r="E196" s="5" t="inlineStr">
+        <is>
+          <t>تسيير الموردين، تسيير مقدمي الخدمات / Gestion des fournisseurs, gestion des prestataires de services</t>
+        </is>
+      </c>
+      <c r="F196" s="5" t="inlineStr">
+        <is>
+          <t>الموردون، مقدمو الخدمات / Fournisseurs, prestataires de services</t>
+        </is>
+      </c>
+      <c r="G196" s="5" t="inlineStr">
+        <is>
+          <t>رقم التعريف الوطني، الاسم واللقب، عنوان البريد الإلكتروني، رقم الهاتف، العنوان، الوظيفة، التسمية الاجتماعية، البنك، رقم الحساب البنكي / NIN, nom et prénom, e-mail, téléphone, adresse, fonction, dénomination sociale, banque, n° compte bancaire</t>
+        </is>
+      </c>
+      <c r="H196" s="5" t="inlineStr">
+        <is>
+          <t>120 شهر (10 سنوات) / 120 mois (10 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" ht="60" customHeight="1">
+      <c r="A197" s="4" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" s="5" t="inlineStr">
+        <is>
+          <t>أشغال الطرق / Travaux routiers</t>
+        </is>
+      </c>
+      <c r="C197" s="5" t="inlineStr">
+        <is>
+          <t>تسيير أوامر بالمهمة / Gestion des ordres de mission</t>
+        </is>
+      </c>
+      <c r="D197" s="5" t="inlineStr">
+        <is>
+          <t>تفويض وضمان سلامة التنقل المهني للعمال / Autoriser et assurer la sécurité des déplacements professionnels des travailleurs</t>
+        </is>
+      </c>
+      <c r="E197" s="5" t="inlineStr">
+        <is>
+          <t>تسيير الأوامر بمهمة / Gestion des ordres de mission</t>
+        </is>
+      </c>
+      <c r="F197" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G197" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، الوظيفة / Nom et prénom, fonction</t>
+        </is>
+      </c>
+      <c r="H197" s="5" t="inlineStr">
+        <is>
+          <t>42 شهر (03 سنوات و06 أشهر) / 42 mois (3 ans et 6 mois)</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" ht="60" customHeight="1">
+      <c r="A198" s="4" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" s="5" t="inlineStr">
+        <is>
+          <t>أشغال الطرق / Travaux routiers</t>
+        </is>
+      </c>
+      <c r="C198" s="5" t="inlineStr">
+        <is>
+          <t>لجنة المشاركة والخدمات الاجتماعية / Comité de participation et des œuvres sociales</t>
+        </is>
+      </c>
+      <c r="D198" s="5" t="inlineStr">
+        <is>
+          <t>تحسين الحالة الاجتماعية للعمال وذوي الحقوق / Amélioration de la situation sociale des travailleurs et ayants droit</t>
+        </is>
+      </c>
+      <c r="E198" s="5" t="inlineStr">
+        <is>
+          <t>تسيير الخدمات الاجتماعية / Gestion des œuvres sociales</t>
+        </is>
+      </c>
+      <c r="F198" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G198" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، تاريخ ومكان الازدياد، الحالة العائلية، عنوان السكن، رقم الهاتف / Nom et prénom, date et lieu de naissance, situation familiale, adresse, téléphone</t>
+        </is>
+      </c>
+      <c r="H198" s="5" t="inlineStr">
+        <is>
+          <t>42 شهر (03 سنوات و06 أشهر) / 42 mois (3 ans et 6 mois)</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" ht="73" customHeight="1">
+      <c r="A199" s="4" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" s="5" t="inlineStr">
+        <is>
+          <t>أشغال الطرق / Travaux routiers</t>
+        </is>
+      </c>
+      <c r="C199" s="5" t="inlineStr">
+        <is>
+          <t>إدارة المشتريات / Gestion des achats</t>
+        </is>
+      </c>
+      <c r="D199" s="5" t="inlineStr">
+        <is>
+          <t>إدارة الطلبات واقتناء المواد الأولية والاستهلاكية والخدمات المختلفة / Gestion des commandes et acquisition des matières premières, consommables et divers services</t>
+        </is>
+      </c>
+      <c r="E199" s="5" t="inlineStr">
+        <is>
+          <t>تسيير المشتريات / Gestion des achats</t>
+        </is>
+      </c>
+      <c r="F199" s="5" t="inlineStr">
+        <is>
+          <t>الموردون / Fournisseurs</t>
+        </is>
+      </c>
+      <c r="G199" s="5" t="inlineStr">
+        <is>
+          <t>رقم التعريف الوطني، الاسم واللقب، عنوان البريد الإلكتروني، رقم الهاتف، العنوان، البنك، رقم الحساب البنكي، رخصة السياقة / NIN, nom et prénom, e-mail, téléphone, adresse, banque, n° compte bancaire, permis de conduire</t>
+        </is>
+      </c>
+      <c r="H199" s="5" t="inlineStr">
+        <is>
+          <t>180 شهر (15 سنة) / 180 mois (15 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" ht="138" customHeight="1">
+      <c r="A200" s="4" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" s="5" t="inlineStr">
+        <is>
+          <t>أشغال عمومية / Travaux publics</t>
+        </is>
+      </c>
+      <c r="C200" s="5" t="inlineStr">
+        <is>
+          <t>إدارة شؤون العمال / Gestion du personnel</t>
+        </is>
+      </c>
+      <c r="D200" s="5" t="inlineStr">
+        <is>
+          <t>إدارة العمال / Gestion des travailleurs</t>
+        </is>
+      </c>
+      <c r="E200" s="5" t="inlineStr">
+        <is>
+          <t>تسيير المستخدمين / Gestion du personnel</t>
+        </is>
+      </c>
+      <c r="F200" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G200" s="5" t="inlineStr">
+        <is>
+          <t>رقم التعريف الوطني، الاسم واللقب، تاريخ ومكان الازدياد، الحالة العائلية، صورة، معطيات بيومترية، عنوان السكن، عنوان البريد الإلكتروني، رقم الهاتف، رقم وثيقة الهوية/رخصة السياقة/جواز السفر، رقم الضمان الاجتماعي، السيرة الذاتية، الراتب، البنك-البريد، رقم الحساب البريدي والبنكي / NIN, nom et prénom, date et lieu de naissance, situation familiale, photo, données biométriques, adresse, e-mail, téléphone, n° CNI/permis de conduire/passeport, n° sécurité sociale, CV, salaire, banque-poste, n° compte postal et bancaire</t>
+        </is>
+      </c>
+      <c r="H200" s="5" t="inlineStr">
+        <is>
+          <t>384 شهر (32 سنة) / 384 mois (32 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" ht="73" customHeight="1">
+      <c r="A201" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" s="5" t="inlineStr">
+        <is>
+          <t>الصناعة الغذائية / Industrie alimentaire</t>
+        </is>
+      </c>
+      <c r="C201" s="5" t="inlineStr">
+        <is>
+          <t>التوعية والسلامة الصحية والمهنية لفائدة الموظفين / Sensibilisation et sécurité sanitaire et professionnelle au profit des employés</t>
+        </is>
+      </c>
+      <c r="D201" s="5" t="inlineStr">
+        <is>
+          <t>إثراء ثقافة السلامة لدى الموظفين، ضمان حماية الموظفين في مكان العمل / Enrichir la culture de sécurité chez les employés et assurer leur protection sur le lieu de travail</t>
+        </is>
+      </c>
+      <c r="E201" s="5" t="inlineStr">
+        <is>
+          <t>تسيير الصحة والسلامة المهنية والبيئة / Gestion de la santé, de la sécurité au travail et de l'environnement</t>
+        </is>
+      </c>
+      <c r="F201" s="5" t="inlineStr">
+        <is>
+          <t>مقدمو الخدمات / Prestataires de services</t>
+        </is>
+      </c>
+      <c r="G201" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، صورة، الوظيفة، الرتبة، رقم التسجيل / Nom et prénom, photo, fonction, grade, matricule</t>
+        </is>
+      </c>
+      <c r="H201" s="5" t="inlineStr">
+        <is>
+          <t>120 شهر (10 سنوات) / 120 mois (10 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" ht="112" customHeight="1">
+      <c r="A202" s="4" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" s="5" t="inlineStr">
+        <is>
+          <t>الصناعة الغذائية / Industrie alimentaire</t>
+        </is>
+      </c>
+      <c r="C202" s="5" t="inlineStr">
+        <is>
+          <t>تسيير الخدمات الاجتماعية / Gestion des œuvres sociales</t>
+        </is>
+      </c>
+      <c r="D202" s="5" t="inlineStr">
+        <is>
+          <t>مساعدة الموظفين وذوي الحقوق على تقليل جزء من نفقاتهم المتعلقة بأمراضهم الخطيرة، تعزيز التزامات الموظفين وتعزيز تماسك الفريق / Aider les employés et ayants droit à réduire une partie de leurs dépenses liées à des maladies graves, renforcer l'engagement des employés et la cohésion d'équipe</t>
+        </is>
+      </c>
+      <c r="E202" s="5" t="inlineStr">
+        <is>
+          <t>تسيير الخدمات الاجتماعية / Gestion des œuvres sociales</t>
+        </is>
+      </c>
+      <c r="F202" s="5" t="inlineStr">
+        <is>
+          <t>ذوو حقوق الأجير (الزوج(ة) والأبناء) / Ayants droit du salarié (conjoint et enfants)</t>
+        </is>
+      </c>
+      <c r="G202" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، تاريخ ومكان الازدياد، الحالة العائلية، رقم الهاتف، الوظيفة، الرتبة، رقم التسجيل، الهيكل التنظيمي التابع لها، رأي الطبيب، الدخل، كشف الهوية البنكية / Nom et prénom, date et lieu de naissance, situation familiale, téléphone, fonction, grade, matricule, structure organisationnelle de rattachement, avis du médecin, revenu, relevé d'identité bancaire</t>
+        </is>
+      </c>
+      <c r="H202" s="5" t="inlineStr">
+        <is>
+          <t>180 شهر (15 سنة) / 180 mois (15 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" ht="60" customHeight="1">
+      <c r="A203" s="4" t="n">
+        <v>202</v>
+      </c>
+      <c r="B203" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C203" s="5" t="inlineStr">
+        <is>
+          <t>استشارة عروض السوق / Consultation des offres du marché</t>
+        </is>
+      </c>
+      <c r="D203" s="5" t="inlineStr">
+        <is>
+          <t>تحليل وتقييم عروض السوق / Analyse et évaluation des offres du marché</t>
+        </is>
+      </c>
+      <c r="E203" s="5" t="inlineStr">
+        <is>
+          <t>استشارة السوق / Consultation du marché</t>
+        </is>
+      </c>
+      <c r="F203" s="5" t="inlineStr">
+        <is>
+          <t>المتعهدون / Soumissionnaires</t>
+        </is>
+      </c>
+      <c r="G203" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، عنوان البريد الإلكتروني، رقم الهاتف، التوقيع، رقم السجل التجاري / Nom et prénom, e-mail, téléphone, signature, n° registre de commerce</t>
+        </is>
+      </c>
+      <c r="H203" s="5" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" ht="99" customHeight="1">
+      <c r="A204" s="4" t="n">
+        <v>203</v>
+      </c>
+      <c r="B204" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C204" s="5" t="inlineStr">
+        <is>
+          <t>إدارة الخبراء والاستشاريين / Gestion des experts et consultants</t>
+        </is>
+      </c>
+      <c r="D204" s="5" t="inlineStr">
+        <is>
+          <t>إدارة تدخلات ومهام الخبراء والاستشاريين / Gestion des interventions et missions des experts et consultants</t>
+        </is>
+      </c>
+      <c r="E204" s="5" t="inlineStr">
+        <is>
+          <t>تسيير الخبراء والاستشاريين / Gestion des experts et consultants</t>
+        </is>
+      </c>
+      <c r="F204" s="5" t="inlineStr">
+        <is>
+          <t>الاستشاريون، الخبراء / Consultants, experts</t>
+        </is>
+      </c>
+      <c r="G204" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، عنوان السكن، عنوان البريد الإلكتروني، رقم الهاتف، التوقيع، رقم وثيقة الهوية/رخصة السياقة/جواز السفر، نسخة من بطاقة المقاول الذاتي، السيرة الذاتية، الحساب البنكي / Nom et prénom, adresse, e-mail, téléphone, signature, n° CNI/permis de conduire/passeport, copie de la carte d'auto-entrepreneur, CV, compte bancaire</t>
+        </is>
+      </c>
+      <c r="H204" s="5" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" ht="60" customHeight="1">
+      <c r="A205" s="4" t="n">
+        <v>204</v>
+      </c>
+      <c r="B205" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C205" s="5" t="inlineStr">
+        <is>
+          <t>حماية الموقع / Protection du site</t>
+        </is>
+      </c>
+      <c r="D205" s="5" t="inlineStr">
+        <is>
+          <t>ضمان أمن الموقع وممتلكات الشركة / Assurer la sécurité du site et des biens de l'entreprise</t>
+        </is>
+      </c>
+      <c r="E205" s="5" t="inlineStr">
+        <is>
+          <t>حماية الموقع / Protection du site</t>
+        </is>
+      </c>
+      <c r="F205" s="5" t="inlineStr">
+        <is>
+          <t>الموردون، الزوار، الزبائن الحاليون أو المحتملون / Fournisseurs, visiteurs, clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G205" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، رقم وثيقة الهوية/رخصة السياقة/جواز السفر، نوع المركبة، ترقيم المركبة / Nom et prénom, n° CNI/permis de conduire/passeport, type de véhicule, immatriculation du véhicule</t>
+        </is>
+      </c>
+      <c r="H205" s="5" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" ht="60" customHeight="1">
+      <c r="A206" s="4" t="n">
+        <v>205</v>
+      </c>
+      <c r="B206" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C206" s="5" t="inlineStr">
+        <is>
+          <t>إدارة شكاوى العملاء / Gestion des réclamations des clients</t>
+        </is>
+      </c>
+      <c r="D206" s="5" t="inlineStr">
+        <is>
+          <t>تسجيل ومعالجة شكاوى العملاء / Enregistrement et traitement des réclamations des clients</t>
+        </is>
+      </c>
+      <c r="E206" s="5" t="inlineStr">
+        <is>
+          <t>تسيير شكاوى الزبائن / Gestion des réclamations des clients</t>
+        </is>
+      </c>
+      <c r="F206" s="5" t="inlineStr">
+        <is>
+          <t>الزبائن الحاليون أو المحتملون / Clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G206" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، عنوان البريد الإلكتروني، رقم الهاتف، عنوان السكن، التوقيع، رقم السجل التجاري / Nom et prénom, e-mail, téléphone, adresse, signature, n° registre de commerce</t>
+        </is>
+      </c>
+      <c r="H206" s="5" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" ht="60" customHeight="1">
+      <c r="A207" s="4" t="n">
+        <v>206</v>
+      </c>
+      <c r="B207" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C207" s="5" t="inlineStr">
+        <is>
+          <t>إدارة التسويق التشغيلي / Gestion du marketing opérationnel</t>
+        </is>
+      </c>
+      <c r="D207" s="5" t="inlineStr">
+        <is>
+          <t>تنفيذ الأنشطة التسويقية الميدانية / Mise en œuvre des activités marketing sur le terrain</t>
+        </is>
+      </c>
+      <c r="E207" s="5" t="inlineStr">
+        <is>
+          <t>تسيير التسويق التشغيلي / Gestion du marketing opérationnel</t>
+        </is>
+      </c>
+      <c r="F207" s="5" t="inlineStr">
+        <is>
+          <t>الزبائن الحاليون أو المحتملون / Clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G207" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، عنوان البريد الإلكتروني، رقم الهاتف، التوقيع، صورة / Nom et prénom, e-mail, téléphone, signature, photo</t>
+        </is>
+      </c>
+      <c r="H207" s="5" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" ht="138" customHeight="1">
+      <c r="A208" s="4" t="n">
+        <v>207</v>
+      </c>
+      <c r="B208" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C208" s="5" t="inlineStr">
+        <is>
+          <t>توظيف واختيار المرشحين / Recrutement et sélection des candidats</t>
+        </is>
+      </c>
+      <c r="D208" s="5" t="inlineStr">
+        <is>
+          <t>استقطاب وتقييم وتوظيف المرشحين / Attirer, évaluer et recruter les candidats</t>
+        </is>
+      </c>
+      <c r="E208" s="5" t="inlineStr">
+        <is>
+          <t>تسيير التوظيف / Gestion du recrutement</t>
+        </is>
+      </c>
+      <c r="F208" s="5" t="inlineStr">
+        <is>
+          <t>المرشحون / Candidats</t>
+        </is>
+      </c>
+      <c r="G208" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، رقم الهاتف، عنوان البريد الإلكتروني، صحيفة السوابق القضائية، استمارة الوكالة الوطنية للتشغيل، السيرة الذاتية / Nom et prénom, téléphone, e-mail, casier judiciaire, formulaire de l'Agence nationale de l'emploi, CV</t>
+        </is>
+      </c>
+      <c r="H208" s="5" t="inlineStr">
+        <is>
+          <t>12 شهر بالنسبة للاسم واللقب، رقم الهاتف، عنوان البريد الإلكتروني، استمارة الوكالة الوطنية للتشغيل والسيرة الذاتية؛ 0 شهر بالنسبة لصحيفة السوابق القضائية / 12 mois pour nom et prénom, téléphone, e-mail, formulaire ANEM et CV ; 0 mois pour le casier judiciaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" ht="73" customHeight="1">
+      <c r="A209" s="4" t="n">
+        <v>208</v>
+      </c>
+      <c r="B209" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C209" s="5" t="inlineStr">
+        <is>
+          <t>إدارة الموردين / Gestion des fournisseurs</t>
+        </is>
+      </c>
+      <c r="D209" s="5" t="inlineStr">
+        <is>
+          <t>إدارة الموردين وضمان جودة التوريدات وتوافقها واستمراريتها / Gestion des fournisseurs et garantie de la qualité, de la conformité et de la continuité des approvisionnements</t>
+        </is>
+      </c>
+      <c r="E209" s="5" t="inlineStr">
+        <is>
+          <t>تسيير الموردين / Gestion des fournisseurs</t>
+        </is>
+      </c>
+      <c r="F209" s="5" t="inlineStr">
+        <is>
+          <t>الموردون / Fournisseurs</t>
+        </is>
+      </c>
+      <c r="G209" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، عنوان البريد الإلكتروني، رقم الهاتف، رقم وثيقة الهوية/رخصة السياقة/جواز السفر، التوقيع، رقم السجل التجاري، الحساب البنكي / Nom et prénom, e-mail, téléphone, n° CNI/permis de conduire/passeport, signature, n° registre de commerce, compte bancaire</t>
+        </is>
+      </c>
+      <c r="H209" s="5" t="inlineStr">
+        <is>
+          <t>120 شهر (10 سنوات) / 120 mois (10 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" ht="73" customHeight="1">
+      <c r="A210" s="4" t="n">
+        <v>209</v>
+      </c>
+      <c r="B210" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C210" s="5" t="inlineStr">
+        <is>
+          <t>إدارة الحملات الترويجية وحملات السحب / Gestion des campagnes promotionnelles et des tirages au sort</t>
+        </is>
+      </c>
+      <c r="D210" s="5" t="inlineStr">
+        <is>
+          <t>تخطيط وتنظيم وتنسيق الأنشطة التسويقية الهادفة إلى جذب انتباه العملاء / Planification, organisation et coordination des activités marketing visant à attirer l'attention des clients</t>
+        </is>
+      </c>
+      <c r="E210" s="5" t="inlineStr">
+        <is>
+          <t>تسيير الحملات الترويجية وحملات السحب / Gestion des campagnes promotionnelles et des tirages au sort</t>
+        </is>
+      </c>
+      <c r="F210" s="5" t="inlineStr">
+        <is>
+          <t>الزبائن الحاليون أو المحتملون / Clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G210" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، عنوان السكن، عنوان البريد الإلكتروني / Nom et prénom, adresse, e-mail (liste partiellement visible sur le document)</t>
+        </is>
+      </c>
+      <c r="H210" s="5" t="inlineStr">
+        <is>
+          <t>غير ظاهرة على الوثيقة / Non visible sur le document</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" ht="99" customHeight="1">
+      <c r="A211" s="4" t="n">
+        <v>210</v>
+      </c>
+      <c r="B211" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C211" s="5" t="inlineStr">
+        <is>
+          <t>تسيير المتمهنين / Gestion des apprentis</t>
+        </is>
+      </c>
+      <c r="D211" s="5" t="inlineStr">
+        <is>
+          <t>متابعة وتأطير تكوين المتمهنين / Suivi et encadrement de la formation des apprentis</t>
+        </is>
+      </c>
+      <c r="E211" s="5" t="inlineStr">
+        <is>
+          <t>تسيير المتمهنين / Gestion des apprentis</t>
+        </is>
+      </c>
+      <c r="F211" s="5" t="inlineStr">
+        <is>
+          <t>المتمهنون / Apprentis</t>
+        </is>
+      </c>
+      <c r="G211" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، تاريخ الازدياد، رقم وثيقة الهوية/رخصة السياقة/جواز السفر، صورة، عنوان السكن، رقم الهاتف، التوقيع، نسخة من بطاقة الهوية الوطنية، الحساب البنكي / Nom et prénom, date de naissance, n° CNI/permis de conduire/passeport, photo, adresse, téléphone, signature, copie de la carte d'identité nationale, compte bancaire</t>
+        </is>
+      </c>
+      <c r="H211" s="5" t="inlineStr">
+        <is>
+          <t>36 شهر (03 سنوات) / 36 mois (3 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" ht="60" customHeight="1">
+      <c r="A212" s="4" t="n">
+        <v>211</v>
+      </c>
+      <c r="B212" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C212" s="5" t="inlineStr">
+        <is>
+          <t>إعداد التقارير / Élaboration des rapports</t>
+        </is>
+      </c>
+      <c r="D212" s="5" t="inlineStr">
+        <is>
+          <t>ضمان إعداد التقارير وتقديمها إلى مجلس الإدارة والمجمع / Assurer l'élaboration des rapports et leur présentation au conseil d'administration et au groupe</t>
+        </is>
+      </c>
+      <c r="E212" s="5" t="inlineStr">
+        <is>
+          <t>إعداد وتقديم التقارير / Élaboration et présentation des rapports</t>
+        </is>
+      </c>
+      <c r="F212" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء، الموردون، الزبائن الحاليون أو المحتملون / Salariés, fournisseurs, clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G212" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، رقم السجل التجاري، الوظيفة، الدخل / Nom et prénom, n° registre de commerce, fonction, revenu</t>
+        </is>
+      </c>
+      <c r="H212" s="5" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" ht="60" customHeight="1">
+      <c r="A213" s="4" t="n">
+        <v>212</v>
+      </c>
+      <c r="B213" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C213" s="5" t="inlineStr">
+        <is>
+          <t>إدارة الفعاليات / Gestion des événements</t>
+        </is>
+      </c>
+      <c r="D213" s="5" t="inlineStr">
+        <is>
+          <t>تنظيم وتنسيق الفعاليات الداخلية والخارجية / Organisation et coordination des événements internes et externes</t>
+        </is>
+      </c>
+      <c r="E213" s="5" t="inlineStr">
+        <is>
+          <t>تسيير الفعاليات / Gestion des événements</t>
+        </is>
+      </c>
+      <c r="F213" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء، الزبائن الحاليون أو المحتملون / Salariés, clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G213" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، رقم الهاتف، التوقيع، الوظيفة / Nom et prénom, téléphone, signature, fonction</t>
+        </is>
+      </c>
+      <c r="H213" s="5" t="inlineStr">
+        <is>
+          <t>03 أشهر / 3 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="214" ht="73" customHeight="1">
+      <c r="A214" s="4" t="n">
+        <v>213</v>
+      </c>
+      <c r="B214" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C214" s="5" t="inlineStr">
+        <is>
+          <t>الإدارة التجارية / Administration commerciale</t>
+        </is>
+      </c>
+      <c r="D214" s="5" t="inlineStr">
+        <is>
+          <t>تطوير وإدارة الأنشطة التجارية / Développement et gestion des activités commerciales</t>
+        </is>
+      </c>
+      <c r="E214" s="5" t="inlineStr">
+        <is>
+          <t>تسيير الزبائن / Gestion des clients</t>
+        </is>
+      </c>
+      <c r="F214" s="5" t="inlineStr">
+        <is>
+          <t>الزبائن الحاليون أو المحتملون / Clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G214" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، عنوان السكن، رقم الهاتف، رقم وثيقة الهوية/رخصة السياقة/جواز السفر، التوقيع، رقم السجل التجاري، عنوان البريد الإلكتروني / Nom et prénom, adresse, téléphone, n° CNI/permis de conduire/passeport, signature, n° registre de commerce, e-mail</t>
+        </is>
+      </c>
+      <c r="H214" s="5" t="inlineStr">
+        <is>
+          <t>120 شهر (10 سنوات) / 120 mois (10 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" ht="60" customHeight="1">
+      <c r="A215" s="4" t="n">
+        <v>214</v>
+      </c>
+      <c r="B215" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C215" s="5" t="inlineStr">
+        <is>
+          <t>تكييف منصب العمل / Adaptation du poste de travail</t>
+        </is>
+      </c>
+      <c r="D215" s="5" t="inlineStr">
+        <is>
+          <t>تكييف المنصب حسب احتياجات الصحة والسلامة / Adaptation du poste selon les besoins de santé et de sécurité</t>
+        </is>
+      </c>
+      <c r="E215" s="5" t="inlineStr">
+        <is>
+          <t>تكييف منصب العمل / Adaptation du poste de travail</t>
+        </is>
+      </c>
+      <c r="F215" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G215" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، شهادة طبية لتكييف المنصب، الوظيفة / Nom et prénom, certificat médical d'adaptation du poste, fonction</t>
+        </is>
+      </c>
+      <c r="H215" s="5" t="inlineStr">
+        <is>
+          <t>384 شهر (32 سنة) / 384 mois (32 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" ht="60" customHeight="1">
+      <c r="A216" s="4" t="n">
+        <v>215</v>
+      </c>
+      <c r="B216" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C216" s="5" t="inlineStr">
+        <is>
+          <t>المراقبة بالفيديو / Vidéosurveillance</t>
+        </is>
+      </c>
+      <c r="D216" s="5" t="inlineStr">
+        <is>
+          <t>ضمان أمن الموقع وممتلكات الشركة / Assurer la sécurité du site et des biens de l'entreprise</t>
+        </is>
+      </c>
+      <c r="E216" s="5" t="inlineStr">
+        <is>
+          <t>المراقبة عن طريق الفيديو / Surveillance par vidéo</t>
+        </is>
+      </c>
+      <c r="F216" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء، الموردون، الزوار، الزبائن الحاليون أو المحتملون / Salariés, fournisseurs, visiteurs, clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G216" s="5" t="inlineStr">
+        <is>
+          <t>صور الفيديو / Images vidéo</t>
+        </is>
+      </c>
+      <c r="H216" s="5" t="inlineStr">
+        <is>
+          <t>01 شهر / 1 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="217" ht="60" customHeight="1">
+      <c r="A217" s="4" t="n">
+        <v>216</v>
+      </c>
+      <c r="B217" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C217" s="5" t="inlineStr">
+        <is>
+          <t>لجنة التأديب / Commission de discipline</t>
+        </is>
+      </c>
+      <c r="D217" s="5" t="inlineStr">
+        <is>
+          <t>دراسة ومعاقبة المخالفات التأديبية / Examen et sanction des infractions disciplinaires</t>
+        </is>
+      </c>
+      <c r="E217" s="5" t="inlineStr">
+        <is>
+          <t>اللجان التأديبية / Commissions disciplinaires</t>
+        </is>
+      </c>
+      <c r="F217" s="5" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G217" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، التوقيع، الوظيفة / Nom et prénom, signature, fonction</t>
+        </is>
+      </c>
+      <c r="H217" s="5" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" ht="60" customHeight="1">
+      <c r="A218" s="4" t="n">
+        <v>217</v>
+      </c>
+      <c r="B218" s="5" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C218" s="5" t="inlineStr">
+        <is>
+          <t>الاستمارة والخدمات الإلكترونية / Formulaires et services électroniques</t>
+        </is>
+      </c>
+      <c r="D218" s="5" t="inlineStr">
+        <is>
+          <t>توفير الخدمات والنماذج عبر الإنترنت / Fourniture de services et de formulaires en ligne</t>
+        </is>
+      </c>
+      <c r="E218" s="5" t="inlineStr">
+        <is>
+          <t>الاستمارة والخدمات الإلكترونية / Formulaires et services électroniques</t>
+        </is>
+      </c>
+      <c r="F218" s="5" t="inlineStr">
+        <is>
+          <t>الزبائن الحاليون أو المحتملون / Clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G218" s="5" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، عنوان البريد الإلكتروني / Nom et prénom, e-mail</t>
+        </is>
+      </c>
+      <c r="H218" s="5" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" ht="60" customHeight="1">
+      <c r="A219" s="2" t="n">
+        <v>218</v>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>إدارة معدات الحماية الفردية / Gestion des équipements de protection individuelle</t>
+        </is>
+      </c>
+      <c r="D219" s="3" t="inlineStr">
+        <is>
+          <t>توفير ومراقبة استخدام معدات الحماية الفردية / Fourniture et contrôle de l'utilisation des équipements de protection individuelle</t>
+        </is>
+      </c>
+      <c r="E219" s="3" t="inlineStr">
+        <is>
+          <t>تسيير معدات الحماية الفردية / Gestion des équipements de protection individuelle</t>
+        </is>
+      </c>
+      <c r="F219" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G219" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، التوقيع، الطول، المقاس / Nom et prénom, signature, taille, mensurations</t>
+        </is>
+      </c>
+      <c r="H219" s="3" t="inlineStr">
+        <is>
+          <t>24 شهر (سنتين) / 24 mois (2 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" ht="60" customHeight="1">
+      <c r="A220" s="2" t="n">
+        <v>219</v>
+      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="inlineStr">
+        <is>
+          <t>إدارة المخزون / Gestion des stocks</t>
+        </is>
+      </c>
+      <c r="D220" s="3" t="inlineStr">
+        <is>
+          <t>مراقبة وتحسين مخزون الشركة / Contrôle et optimisation des stocks de l'entreprise</t>
+        </is>
+      </c>
+      <c r="E220" s="3" t="inlineStr">
+        <is>
+          <t>تسيير المخزون / Gestion des stocks</t>
+        </is>
+      </c>
+      <c r="F220" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء، الموردون / Salariés, fournisseurs</t>
+        </is>
+      </c>
+      <c r="G220" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، التوقيع / Nom et prénom, signature</t>
+        </is>
+      </c>
+      <c r="H220" s="3" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="221" ht="60" customHeight="1">
+      <c r="A221" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="B221" s="3" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C221" s="3" t="inlineStr">
+        <is>
+          <t>اللجنة المشتركة للصحة والسلامة / Commission paritaire de santé et de sécurité</t>
+        </is>
+      </c>
+      <c r="D221" s="3" t="inlineStr">
+        <is>
+          <t>تحسين شروط النظافة والسلامة في العمل / Amélioration des conditions d'hygiène et de sécurité au travail</t>
+        </is>
+      </c>
+      <c r="E221" s="3" t="inlineStr">
+        <is>
+          <t>اللجنة المشتركة للصحة والسلامة / Commission paritaire de santé et de sécurité</t>
+        </is>
+      </c>
+      <c r="F221" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G221" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، التوقيع، الوظيفة / Nom et prénom, signature, fonction</t>
+        </is>
+      </c>
+      <c r="H221" s="3" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="222" ht="60" customHeight="1">
+      <c r="A222" s="2" t="n">
+        <v>221</v>
+      </c>
+      <c r="B222" s="3" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C222" s="3" t="inlineStr">
+        <is>
+          <t>تحصيل ديون العملاء / Recouvrement des créances clients</t>
+        </is>
+      </c>
+      <c r="D222" s="3" t="inlineStr">
+        <is>
+          <t>متابعة واسترجاع الديون من العملاء / Suivi et recouvrement des créances auprès des clients</t>
+        </is>
+      </c>
+      <c r="E222" s="3" t="inlineStr">
+        <is>
+          <t>تحصيل ديون الزبائن / Recouvrement des créances des clients</t>
+        </is>
+      </c>
+      <c r="F222" s="3" t="inlineStr">
+        <is>
+          <t>الزبائن الحاليون أو المحتملون / Clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G222" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، عنوان البريد الإلكتروني، رقم الهاتف، التوقيع، رقم السجل التجاري / Nom et prénom, e-mail, téléphone, signature, n° registre de commerce</t>
+        </is>
+      </c>
+      <c r="H222" s="3" t="inlineStr">
+        <is>
+          <t>120 شهر (10 سنوات) / 120 mois (10 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" ht="60" customHeight="1">
+      <c r="A223" s="2" t="n">
+        <v>222</v>
+      </c>
+      <c r="B223" s="3" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C223" s="3" t="inlineStr">
+        <is>
+          <t>إدارة صندوق التحصيل / Gestion de la caisse de recouvrement</t>
+        </is>
+      </c>
+      <c r="D223" s="3" t="inlineStr">
+        <is>
+          <t>تسيير التدفقات المالية للصندوق / Gestion des flux financiers de la caisse</t>
+        </is>
+      </c>
+      <c r="E223" s="3" t="inlineStr">
+        <is>
+          <t>تسيير صندوق التحصيل / Gestion de la caisse de recouvrement</t>
+        </is>
+      </c>
+      <c r="F223" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G223" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، التوقيع / Nom et prénom, signature</t>
+        </is>
+      </c>
+      <c r="H223" s="3" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" ht="60" customHeight="1">
+      <c r="A224" s="2" t="n">
+        <v>223</v>
+      </c>
+      <c r="B224" s="3" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C224" s="3" t="inlineStr">
+        <is>
+          <t>إدارة التسويق الرقمي / Gestion du marketing digital</t>
+        </is>
+      </c>
+      <c r="D224" s="3" t="inlineStr">
+        <is>
+          <t>الترويج للشركة عبر القنوات الرقمية / Promotion de l'entreprise via les canaux numériques</t>
+        </is>
+      </c>
+      <c r="E224" s="3" t="inlineStr">
+        <is>
+          <t>تسيير التسويق الرقمي / Gestion du marketing digital</t>
+        </is>
+      </c>
+      <c r="F224" s="3" t="inlineStr">
+        <is>
+          <t>الزبائن الحاليون أو المحتملون / Clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G224" s="3" t="inlineStr">
+        <is>
+          <t>صورة الفيديو، الصوت / Image vidéo, voix</t>
+        </is>
+      </c>
+      <c r="H224" s="3" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" ht="60" customHeight="1">
+      <c r="A225" s="2" t="n">
+        <v>224</v>
+      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C225" s="3" t="inlineStr">
+        <is>
+          <t>خطة الصيانة / Plan de maintenance</t>
+        </is>
+      </c>
+      <c r="D225" s="3" t="inlineStr">
+        <is>
+          <t>تخطيط وتنفيذ صيانة المعدات / Planification et exécution de la maintenance des équipements</t>
+        </is>
+      </c>
+      <c r="E225" s="3" t="inlineStr">
+        <is>
+          <t>خطة الصيانة / Plan de maintenance</t>
+        </is>
+      </c>
+      <c r="F225" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G225" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، رقم الهاتف، عنوان البريد الإلكتروني، الوظيفة / Nom et prénom, téléphone, e-mail, fonction</t>
+        </is>
+      </c>
+      <c r="H225" s="3" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="226" ht="60" customHeight="1">
+      <c r="A226" s="2" t="n">
+        <v>225</v>
+      </c>
+      <c r="B226" s="3" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C226" s="3" t="inlineStr">
+        <is>
+          <t>أرشيف بيانات العملاء والموردين / Archives des données des clients et fournisseurs</t>
+        </is>
+      </c>
+      <c r="D226" s="3" t="inlineStr">
+        <is>
+          <t>حفظ وتأمين أرشيف البيانات / Conservation et sécurisation des archives de données</t>
+        </is>
+      </c>
+      <c r="E226" s="3" t="inlineStr">
+        <is>
+          <t>أرشيف بيانات الزبائن والموردين / Archives des données des clients et fournisseurs</t>
+        </is>
+      </c>
+      <c r="F226" s="3" t="inlineStr">
+        <is>
+          <t>الموردون، الزبائن الحاليون أو المحتملون / Fournisseurs, clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G226" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، رقم الهاتف، عنوان البريد الإلكتروني، عنوان السكن، رقم السجل التجاري / Nom et prénom, téléphone, e-mail, adresse, n° registre de commerce</t>
+        </is>
+      </c>
+      <c r="H226" s="3" t="inlineStr">
+        <is>
+          <t>120 شهر (10 سنوات) / 120 mois (10 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" ht="73" customHeight="1">
+      <c r="A227" s="2" t="n">
+        <v>226</v>
+      </c>
+      <c r="B227" s="3" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C227" s="3" t="inlineStr">
+        <is>
+          <t>إدارة خدمة الزبائن / Gestion du service client</t>
+        </is>
+      </c>
+      <c r="D227" s="3" t="inlineStr">
+        <is>
+          <t>إدارة تفاعلات المستهلكين لتحسين تجربة العملاء ودعم الأنشطة التسويقية / Gestion des interactions avec les consommateurs pour améliorer l'expérience client et soutenir les activités marketing</t>
+        </is>
+      </c>
+      <c r="E227" s="3" t="inlineStr">
+        <is>
+          <t>تسيير المستهلكين / Gestion des consommateurs</t>
+        </is>
+      </c>
+      <c r="F227" s="3" t="inlineStr">
+        <is>
+          <t>الزبائن الحاليون أو المحتملون / Clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G227" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، رقم الهاتف، عنوان البريد الإلكتروني، عنوان السكن / Nom et prénom, téléphone, e-mail, adresse</t>
+        </is>
+      </c>
+      <c r="H227" s="3" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" ht="60" customHeight="1">
+      <c r="A228" s="2" t="n">
+        <v>227</v>
+      </c>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C228" s="3" t="inlineStr">
+        <is>
+          <t>دراسة السوق وتطوير المنتجات / Étude de marché et développement des produits</t>
+        </is>
+      </c>
+      <c r="D228" s="3" t="inlineStr">
+        <is>
+          <t>تحليل السوق ومدى رضا الزبائن عن المنتجات / Analyse du marché et de la satisfaction des clients à l'égard des produits</t>
+        </is>
+      </c>
+      <c r="E228" s="3" t="inlineStr">
+        <is>
+          <t>تسيير الاستطلاعات ودراسة السوق / Gestion des sondages et des études de marché</t>
+        </is>
+      </c>
+      <c r="F228" s="3" t="inlineStr">
+        <is>
+          <t>الزبائن الحاليون أو المحتملون / Clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G228" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، رقم الهاتف، عنوان البريد الإلكتروني، عنوان السكن، الجنس / Nom et prénom, téléphone, e-mail, adresse, sexe</t>
+        </is>
+      </c>
+      <c r="H228" s="3" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="229" ht="99" customHeight="1">
+      <c r="A229" s="2" t="n">
+        <v>228</v>
+      </c>
+      <c r="B229" s="3" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C229" s="3" t="inlineStr">
+        <is>
+          <t>التمثيلية القانونية / Représentation juridique</t>
+        </is>
+      </c>
+      <c r="D229" s="3" t="inlineStr">
+        <is>
+          <t>تسيير الإجراءات القانونية والتمثيل القانوني للمؤسسة أمام الهيئات المختصة / Gestion des procédures juridiques et représentation légale de l'entreprise devant les instances compétentes</t>
+        </is>
+      </c>
+      <c r="E229" s="3" t="inlineStr">
+        <is>
+          <t>التمثيلية القانونية / Représentation juridique</t>
+        </is>
+      </c>
+      <c r="F229" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء، الموردون، الزبائن الحاليون أو المحتملون / Salariés, fournisseurs, clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G229" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، تاريخ الازدياد، عنوان البريد الإلكتروني، عنوان السكن، رقم الهاتف، رقم وثيقة الهوية/رخصة السياقة/جواز السفر، التوقيع، اسم ولقب الأب، اسم ولقب الأم، رقم السجل التجاري / Nom et prénom, date de naissance, e-mail, adresse, téléphone, n° CNI/permis de conduire/passeport, signature, nom et prénom du père, nom et prénom de la mère, n° registre de commerce</t>
+        </is>
+      </c>
+      <c r="H229" s="3" t="inlineStr">
+        <is>
+          <t>60 شهر (05 سنوات) / 60 mois (5 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="230" ht="60" customHeight="1">
+      <c r="A230" s="2" t="n">
+        <v>229</v>
+      </c>
+      <c r="B230" s="3" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C230" s="3" t="inlineStr">
+        <is>
+          <t>تسيير تطوير الكفاءات / Gestion du développement des compétences</t>
+        </is>
+      </c>
+      <c r="D230" s="3" t="inlineStr">
+        <is>
+          <t>تطوير الكفاءات للعمال عن طريق التكوين / Développement des compétences des travailleurs par la formation</t>
+        </is>
+      </c>
+      <c r="E230" s="3" t="inlineStr">
+        <is>
+          <t>تسيير تطوير الكفاءات / Gestion du développement des compétences</t>
+        </is>
+      </c>
+      <c r="F230" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G230" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، عنوان البريد الإلكتروني، رقم الهاتف، التوقيع، الوظيفة / Nom et prénom, e-mail, téléphone, signature, fonction</t>
+        </is>
+      </c>
+      <c r="H230" s="3" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="125" customHeight="1">
+      <c r="A231" s="2" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" s="3" t="inlineStr">
+        <is>
+          <t>البريد السريع / Courrier express</t>
+        </is>
+      </c>
+      <c r="C231" s="3" t="inlineStr">
+        <is>
+          <t>تتبع المركبات المهنية للشركة عبر نظام تحديد الموقع الجغرافي / Suivi des véhicules professionnels de l'entreprise via un système de géolocalisation</t>
+        </is>
+      </c>
+      <c r="D231" s="3" t="inlineStr">
+        <is>
+          <t>متابعة المركبات المهنية في الوقت الفعلي لتأمين السائقين والممتلكات، تحسين التنقلات وضمان إمكانية التتبع في حال وقوع أي حادث، وفقًا للقانون / Suivi en temps réel des véhicules professionnels afin de sécuriser les conducteurs et les biens, d'optimiser les déplacements et de garantir la traçabilité en cas d'accident, conformément à la loi</t>
+        </is>
+      </c>
+      <c r="E231" s="3" t="inlineStr">
+        <is>
+          <t>تسيير الموارد المهنية (أسطول المركبات) / Gestion des ressources professionnelles (flotte de véhicules)</t>
+        </is>
+      </c>
+      <c r="F231" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء، عمال التوصيل المستقلون الذين يستخدمون مركبات الشركة / Salariés, livreurs indépendants utilisant les véhicules de l'entreprise</t>
+        </is>
+      </c>
+      <c r="G231" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، رقم الهاتف، الإحداثيات الجغرافية، رقم التسجيل، ساعات السياقة وفترات الراحة، الرحلات المنجزة، الوضعية المهنية (موظف/عامل توصيل مستقل)، علامة المركبة / Nom et prénom, téléphone, coordonnées géographiques, matricule, heures de conduite et périodes de repos, trajets effectués, statut professionnel (employé/livreur indépendant), marque du véhicule</t>
+        </is>
+      </c>
+      <c r="H231" s="3" t="inlineStr">
+        <is>
+          <t>24 شهر (سنتين) / 24 mois (2 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="190" customHeight="1">
+      <c r="A232" s="2" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" s="3" t="inlineStr">
+        <is>
+          <t>البريد السريع / Courrier express</t>
+        </is>
+      </c>
+      <c r="C232" s="3" t="inlineStr">
+        <is>
+          <t>إدارة الإجراءات التأديبية والنزاعات الخاصة بالموظفين / Gestion des procédures disciplinaires et des litiges relatifs aux employés</t>
+        </is>
+      </c>
+      <c r="D232" s="3" t="inlineStr">
+        <is>
+          <t>ضمان متابعة وإدارة وتتبع الإجراءات التأديبية والنزاعات المتعلقة بالموظفين وفقًا لتشريع العمل والتنظيم الداخلي / Assurer le suivi, la gestion et la traçabilité des procédures disciplinaires et des litiges relatifs aux employés conformément à la législation du travail et au règlement intérieur</t>
+        </is>
+      </c>
+      <c r="E232" s="3" t="inlineStr">
+        <is>
+          <t>تسيير المستخدمين / Gestion du personnel</t>
+        </is>
+      </c>
+      <c r="F232" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G232" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، تاريخ ومكان الازدياد، الحالة العائلية، صورة، معطيات بيومترية، عنوان السكن، عنوان البريد الإلكتروني، رقم الهاتف، رقم وثيقة الهوية/رخصة السياقة/جواز السفر، تسجيلات الفيديوهات، التوقيعات، الوثائق التبريرية والأدلة، الوظيفة، مقر التعيين، استمارة تقييم، السوابق التأديبية، الشهادات، تاريخ التوظيف، بطاقة الوصف الوظيفي / Nom et prénom, date et lieu de naissance, situation familiale, photo, données biométriques, adresse, e-mail, téléphone, n° CNI/permis de conduire/passeport, enregistrements vidéo, signatures, pièces justificatives et preuves, fonction, lieu d'affectation, formulaire d'évaluation, antécédents disciplinaires, diplômes, date de recrutement, fiche de poste</t>
+        </is>
+      </c>
+      <c r="H232" s="3" t="inlineStr">
+        <is>
+          <t>120 شهر (10 سنوات) لمعظم المعطيات؛ 12 شهر بالنسبة لتسجيلات الفيديوهات والوثائق التبريرية والأدلة / 120 mois (10 ans) pour la plupart des données ; 12 mois pour les enregistrements vidéo, les pièces justificatives et les preuves</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" ht="86" customHeight="1">
+      <c r="A233" s="2" t="n">
+        <v>232</v>
+      </c>
+      <c r="B233" s="3" t="inlineStr">
+        <is>
+          <t>إنتاج / Production</t>
+        </is>
+      </c>
+      <c r="C233" s="3" t="inlineStr">
+        <is>
+          <t>المعلومات الشخصية للعمال / Informations personnelles des travailleurs</t>
+        </is>
+      </c>
+      <c r="D233" s="3" t="inlineStr">
+        <is>
+          <t>تسيير المستخدمين والأجور / Gestion du personnel et des salaires</t>
+        </is>
+      </c>
+      <c r="E233" s="3" t="inlineStr">
+        <is>
+          <t>تسيير المستخدمين / Gestion du personnel</t>
+        </is>
+      </c>
+      <c r="F233" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G233" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، تاريخ الازدياد، صورة، عنوان السكن، الحالة العائلية، رقم وثيقة الهوية/رخصة السياقة/جواز السفر، الوظيفة، السيرة الذاتية، الحساب البنكي / Nom et prénom, date de naissance, photo, adresse, situation familiale, n° CNI/permis de conduire/passeport, fonction, CV, compte bancaire</t>
+        </is>
+      </c>
+      <c r="H233" s="3" t="inlineStr">
+        <is>
+          <t>504 شهر (42 سنة) / 504 mois (42 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" ht="125" customHeight="1">
+      <c r="A234" s="2" t="n">
+        <v>233</v>
+      </c>
+      <c r="B234" s="3" t="inlineStr">
+        <is>
+          <t>صناعة المنتجات الإلكترونية / Fabrication de produits électroniques</t>
+        </is>
+      </c>
+      <c r="C234" s="3" t="inlineStr">
+        <is>
+          <t>إدارة نظام الجودة، النظافة، السلامة والبيئة / Gestion du système qualité, hygiène, sécurité et environnement</t>
+        </is>
+      </c>
+      <c r="D234" s="3" t="inlineStr">
+        <is>
+          <t>إدارة نظام جودة، نظافة، سلامة وبيئة وفقًا للمعايير الدولية والتشريعات المعمول بها / Gestion d'un système qualité, hygiène, sécurité et environnement conformément aux normes internationales et aux législations en vigueur</t>
+        </is>
+      </c>
+      <c r="E234" s="3" t="inlineStr">
+        <is>
+          <t>مراقبة نظام إدارة الجودة، النظافة، السلامة والبيئة وفقًا للمعايير الدولية والتشريعات المعمول بها / Contrôle du système de management qualité, hygiène, sécurité et environnement conformément aux normes internationales et aux législations en vigueur</t>
+        </is>
+      </c>
+      <c r="F234" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G234" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، عنوان البريد الإلكتروني، تاريخ ومكان الازدياد، الوظيفة / Nom et prénom, e-mail, date et lieu de naissance, fonction</t>
+        </is>
+      </c>
+      <c r="H234" s="3" t="inlineStr">
+        <is>
+          <t>60 شهر (05 سنوات) / 60 mois (5 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" ht="99" customHeight="1">
+      <c r="A235" s="2" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" s="3" t="inlineStr">
+        <is>
+          <t>صناعة المنتجات الإلكترونية / Fabrication de produits électroniques</t>
+        </is>
+      </c>
+      <c r="C235" s="3" t="inlineStr">
+        <is>
+          <t>إدارة نظام المراقبة بالفيديو / Gestion du système de vidéosurveillance</t>
+        </is>
+      </c>
+      <c r="D235" s="3" t="inlineStr">
+        <is>
+          <t>ضمان أمن الأفراد والممتلكات في مقرات الشركة / Assurer la sécurité des personnes et des biens dans les locaux de l'entreprise</t>
+        </is>
+      </c>
+      <c r="E235" s="3" t="inlineStr">
+        <is>
+          <t>الأمن ومراقبة الدخول / Sécurité et contrôle des accès</t>
+        </is>
+      </c>
+      <c r="F235" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء، الموردون، الزبائن الحاليون أو المحتملون، الزوار، وكل شخص آخر يدخل إلى مقرات الشركة / Salariés, fournisseurs, clients actuels ou potentiels, visiteurs et toute autre personne accédant aux locaux de l'entreprise</t>
+        </is>
+      </c>
+      <c r="G235" s="3" t="inlineStr">
+        <is>
+          <t>صورة، رقم لوحة تسجيل المركبة / Image, numéro d'immatriculation du véhicule</t>
+        </is>
+      </c>
+      <c r="H235" s="3" t="inlineStr">
+        <is>
+          <t>شهر واحد / 1 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" ht="125" customHeight="1">
+      <c r="A236" s="2" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" s="3" t="inlineStr">
+        <is>
+          <t>صناعة المنتجات الإلكترونية / Fabrication de produits électroniques</t>
+        </is>
+      </c>
+      <c r="C236" s="3" t="inlineStr">
+        <is>
+          <t>استقطاب الموظفين / Recrutement du personnel</t>
+        </is>
+      </c>
+      <c r="D236" s="3" t="inlineStr">
+        <is>
+          <t>القيام بعملية استقطاب المرشحين لشغل الوظائف الشاغرة، مع ضمان مواءمة مؤهلاتهم وخبراتهم مع متطلبات المناصب المتاحة / Mener le processus de recrutement des candidats pour pourvoir les postes vacants, en veillant à l'adéquation de leurs qualifications et de leur expérience avec les exigences des postes disponibles</t>
+        </is>
+      </c>
+      <c r="E236" s="3" t="inlineStr">
+        <is>
+          <t>إدارة عمليات التوظيف / Gestion des opérations de recrutement</t>
+        </is>
+      </c>
+      <c r="F236" s="3" t="inlineStr">
+        <is>
+          <t>المترشحون / Candidats</t>
+        </is>
+      </c>
+      <c r="G236" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، تاريخ ومكان الازدياد، الحالة العائلية، صورة، عنوان السكن، رقم الهاتف، شهادات الجامعة وشهادات التكوين / Nom et prénom, date et lieu de naissance, situation familiale, photo, adresse, téléphone, diplômes universitaires et attestations de formation</t>
+        </is>
+      </c>
+      <c r="H236" s="3" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="237" ht="112" customHeight="1">
+      <c r="A237" s="2" t="n">
+        <v>236</v>
+      </c>
+      <c r="B237" s="3" t="inlineStr">
+        <is>
+          <t>صناعة الأدوية / Industrie pharmaceutique</t>
+        </is>
+      </c>
+      <c r="C237" s="3" t="inlineStr">
+        <is>
+          <t>المحاسبة وإدارة الخزينة / Comptabilité et gestion de la trésorerie</t>
+        </is>
+      </c>
+      <c r="D237" s="3" t="inlineStr">
+        <is>
+          <t>تسيير المحاسبة والخزينة الخاصة بالمؤسسة / Gestion de la comptabilité et de la trésorerie de l'entreprise</t>
+        </is>
+      </c>
+      <c r="E237" s="3" t="inlineStr">
+        <is>
+          <t>المحاسبة وتسيير الخزينة / Comptabilité et gestion de la trésorerie</t>
+        </is>
+      </c>
+      <c r="F237" s="3" t="inlineStr">
+        <is>
+          <t>الموردون / Fournisseurs</t>
+        </is>
+      </c>
+      <c r="G237" s="3" t="inlineStr">
+        <is>
+          <t>الإسم واللقب، عنوان السكن، عنوان البريد الإلكتروني، رقم الهاتف، رقم وثيقة الهوية/رخصة السياقة/جواز السفر، نسخة من وثيقة الهوية الوطنية، التوقيع، رقم السجل التجاري، الحساب البنكي، رقم التعريف الجبائي / Nom et prénom, adresse, e-mail, téléphone, n° CNI/permis de conduire/passeport, copie de la pièce d'identité nationale, signature, n° registre de commerce, compte bancaire, NIF</t>
+        </is>
+      </c>
+      <c r="H237" s="3" t="inlineStr">
+        <is>
+          <t>120 شهر (10 سنوات) / 120 mois (10 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" ht="125" customHeight="1">
+      <c r="A238" s="2" t="n">
+        <v>237</v>
+      </c>
+      <c r="B238" s="3" t="inlineStr">
+        <is>
+          <t>صناعة الأدوية / Industrie pharmaceutique</t>
+        </is>
+      </c>
+      <c r="C238" s="3" t="inlineStr">
+        <is>
+          <t>إستضافة ومشاركة وحفظ البيانات / Hébergement, partage et conservation des données</t>
+        </is>
+      </c>
+      <c r="D238" s="3" t="inlineStr">
+        <is>
+          <t>إستضافة، مشاركة وحفظ البيانات / Hébergement, partage et conservation des données</t>
+        </is>
+      </c>
+      <c r="E238" s="3" t="inlineStr">
+        <is>
+          <t>تسيير إستضافة المعطيات ومشاركتها وحفظها / Gestion de l'hébergement, du partage et de la conservation des données</t>
+        </is>
+      </c>
+      <c r="F238" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء، الموردون، الزبائن الحاليون أو المحتملون / Salariés, fournisseurs, clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G238" s="3" t="inlineStr">
+        <is>
+          <t>الإسم واللقب، عنوان السكن، عنوان البريد الإلكتروني، رقم الهاتف، معطيات الموارد البشرية (ملفات الأجراء، التقييمات، العطل، الوثائق الإدارية)، المعطيات التقنية (سجلات النظام، معرفات المستخدمين، عناوين بروتوكول الأنترنت الداخلية)، الوظيفة / Nom et prénom, adresse, e-mail, téléphone, données RH (dossiers des salariés, évaluations, congés, documents administratifs), données techniques (journaux système, identifiants utilisateurs, adresses IP internes), fonction</t>
+        </is>
+      </c>
+      <c r="H238" s="3" t="inlineStr">
+        <is>
+          <t>120 شهر (10 سنوات) / 120 mois (10 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" ht="47" customHeight="1">
+      <c r="A239" s="2" t="n">
+        <v>238</v>
+      </c>
+      <c r="B239" s="3" t="inlineStr">
+        <is>
+          <t>صناعة الأدوية / Industrie pharmaceutique</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="inlineStr">
+        <is>
+          <t>الاتصال / Communication</t>
+        </is>
+      </c>
+      <c r="D239" s="3" t="inlineStr">
+        <is>
+          <t>تسهيل وتنظيم الاتصال الداخلي والخارجي / Faciliter et organiser la communication interne et externe</t>
+        </is>
+      </c>
+      <c r="E239" s="3" t="inlineStr">
+        <is>
+          <t>الاتصال / Communication</t>
+        </is>
+      </c>
+      <c r="F239" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء، الزبائن الحاليون أو المحتملون / Salariés, clients actuels ou potentiels</t>
+        </is>
+      </c>
+      <c r="G239" s="3" t="inlineStr">
+        <is>
+          <t>الإسم واللقب، عنوان البريد الإلكتروني، رقم الهاتف، عنوان السكن / Nom et prénom, e-mail, téléphone, adresse</t>
+        </is>
+      </c>
+      <c r="H239" s="3" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="240" ht="47" customHeight="1">
+      <c r="A240" s="2" t="n">
+        <v>239</v>
+      </c>
+      <c r="B240" s="3" t="inlineStr">
+        <is>
+          <t>صناعة الأدوية / Industrie pharmaceutique</t>
+        </is>
+      </c>
+      <c r="C240" s="3" t="inlineStr">
+        <is>
+          <t>اللجنة المشتركة للصحة والسلامة / Commission paritaire de santé et de sécurité</t>
+        </is>
+      </c>
+      <c r="D240" s="3" t="inlineStr">
+        <is>
+          <t>متابعة أعمال اللجنة المشتركة للصحة والسلامة / Suivi des travaux de la commission paritaire de santé et de sécurité</t>
+        </is>
+      </c>
+      <c r="E240" s="3" t="inlineStr">
+        <is>
+          <t>اللجنة المشتركة للصحة والسلامة / Commission paritaire de santé et de sécurité</t>
+        </is>
+      </c>
+      <c r="F240" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G240" s="3" t="inlineStr">
+        <is>
+          <t>الإسم واللقب، التوقيع، الوظيفة / Nom et prénom, signature, fonction</t>
+        </is>
+      </c>
+      <c r="H240" s="3" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="241" ht="86" customHeight="1">
+      <c r="A241" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="B241" s="3" t="inlineStr">
+        <is>
+          <t>صناعة الأدوية / Industrie pharmaceutique</t>
+        </is>
+      </c>
+      <c r="C241" s="3" t="inlineStr">
+        <is>
+          <t>حماية الموقع / Protection du site</t>
+        </is>
+      </c>
+      <c r="D241" s="3" t="inlineStr">
+        <is>
+          <t>ضمان أمن وحماية الموقع / Assurer la sûreté et la protection du site</t>
+        </is>
+      </c>
+      <c r="E241" s="3" t="inlineStr">
+        <is>
+          <t>أمن الموقع / Sécurité du site</t>
+        </is>
+      </c>
+      <c r="F241" s="3" t="inlineStr">
+        <is>
+          <t>الموردون، الزبائن الحاليون أو المحتملون، الزوار / Fournisseurs, clients actuels ou potentiels, visiteurs</t>
+        </is>
+      </c>
+      <c r="G241" s="3" t="inlineStr">
+        <is>
+          <t>الإسم واللقب، رقم وثيقة الهوية/رخصة السياقة/جواز السفر، نوع المركبة، رقم تسجيل المركبة، نسخة من بطاقة الإقامة للأجانب، نسخة من جواز السفر / Nom et prénom, n° CNI/permis de conduire/passeport, type de véhicule, immatriculation du véhicule, copie de la carte de résidence pour les étrangers, copie du passeport</t>
+        </is>
+      </c>
+      <c r="H241" s="3" t="inlineStr">
+        <is>
+          <t>12 شهر / 12 mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="242" ht="99" customHeight="1">
+      <c r="A242" s="2" t="n">
+        <v>241</v>
+      </c>
+      <c r="B242" s="3" t="inlineStr">
+        <is>
+          <t>صناعة المنتجات الصيدلانية / Fabrication de produits pharmaceutiques</t>
+        </is>
+      </c>
+      <c r="C242" s="3" t="inlineStr">
+        <is>
+          <t>تسيير لجنة المشاركة / Gestion du comité de participation</t>
+        </is>
+      </c>
+      <c r="D242" s="3" t="inlineStr">
+        <is>
+          <t>تسيير الخدمات الاجتماعية لفائدة الموظفين من أجل تحسين رفاهيتهم وتعزيز التماسك الاجتماعي داخل المؤسسة / Gestion des œuvres sociales au profit des employés afin d'améliorer leur bien-être et de renforcer la cohésion sociale au sein de l'entreprise</t>
+        </is>
+      </c>
+      <c r="E242" s="3" t="inlineStr">
+        <is>
+          <t>تسيير لجنة المشاركة / Gestion du comité de participation</t>
+        </is>
+      </c>
+      <c r="F242" s="3" t="inlineStr">
+        <is>
+          <t>الأجراء / Salariés</t>
+        </is>
+      </c>
+      <c r="G242" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، تاريخ ومكان الازدياد، شهادة وفاة، جواز السفر، رقم التعريف الوطني، عنوان البريد الإلكتروني، الحساب البنكي، المبلغ / Nom et prénom, date et lieu de naissance, acte de décès, passeport, NIN, e-mail, compte bancaire, montant</t>
+        </is>
+      </c>
+      <c r="H242" s="3" t="inlineStr">
+        <is>
+          <t>384 شهر (32 سنة) / 384 mois (32 ans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="243" ht="99" customHeight="1">
+      <c r="A243" s="2" t="n">
+        <v>242</v>
+      </c>
+      <c r="B243" s="3" t="inlineStr">
+        <is>
+          <t>إنتاج المياه المعدنية ومياه الينابيع / Production d'eaux minérales et d'eaux de source</t>
+        </is>
+      </c>
+      <c r="C243" s="3" t="inlineStr">
+        <is>
+          <t>المحاسبة وإدارة الخزينة / Comptabilité et gestion de la trésorerie</t>
+        </is>
+      </c>
+      <c r="D243" s="3" t="inlineStr">
+        <is>
+          <t>ضمان إدارة مالية فعالة من خلال مراقبة تدفقات الأموال / Assurer une gestion financière efficace par le contrôle des flux de fonds</t>
+        </is>
+      </c>
+      <c r="E243" s="3" t="inlineStr">
+        <is>
+          <t>المحاسبة وتسيير الخزينة / Comptabilité et gestion de la trésorerie</t>
+        </is>
+      </c>
+      <c r="F243" s="3" t="inlineStr">
+        <is>
+          <t>الموردون، أعضاء مجلس الإدارة، المساهمون / Fournisseurs, membres du conseil d'administration, actionnaires</t>
+        </is>
+      </c>
+      <c r="G243" s="3" t="inlineStr">
+        <is>
+          <t>الاسم واللقب، عنوان السكن، عنوان البريد الإلكتروني، رقم الهاتف، رقم وثيقة الهوية/رخصة السياقة/جواز السفر، التوقيع، نسخة من بطاقة الهوية الوطنية، رقم السجل التجاري، الحساب البنكي / Nom et prénom, adresse, e-mail, téléphone, n° CNI/permis de conduire/passeport, signature, copie de la carte d'identité nationale, n° registre de commerce, compte bancaire</t>
+        </is>
+      </c>
+      <c r="H243" s="3" t="inlineStr">
         <is>
           <t>120 شهر (10 سنوات) / 120 mois (10 ans)</t>
         </is>

</xml_diff>